<commit_message>
chore: 更新 DataTable 配置表
- EnemyTable: 更新敌人配置
- SummonChessTable: 更新召唤棋子配置
- 删除临时文件
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/SummonChessTable.xlsx
+++ b/AAAGameData/DataTables/SummonChessTable.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="123">
   <si>
     <t>#</t>
   </si>
@@ -2125,9 +2125,7 @@
       <c r="AC9" s="1">
         <v>0</v>
       </c>
-      <c r="AD9" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="AD9" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: SummonChess棋子系统 - 配置表更新及SummonChessStateUI组件
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/SummonChessTable.xlsx
+++ b/AAAGameData/DataTables/SummonChessTable.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11925"/>
+    <workbookView windowWidth="29868" windowHeight="15300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="128">
   <si>
     <t>#</t>
   </si>
@@ -59,6 +59,9 @@
     <t>IconId</t>
   </si>
   <si>
+    <t>HeadImgId</t>
+  </si>
+  <si>
     <t>MaxHp</t>
   </si>
   <si>
@@ -161,7 +164,10 @@
     <t>棋子预制体资源ID（阶级数组，暂时三阶相同）</t>
   </si>
   <si>
-    <t>UI图标资源ID（阶级数组，暂时三阶相同）</t>
+    <t>棋子图标资源ID（阶级数组，暂时三阶相同）</t>
+  </si>
+  <si>
+    <t>棋子头像资源ID（阶级数组，暂时三阶相同）</t>
   </si>
   <si>
     <t>最大生命值（三个阶级）</t>
@@ -236,7 +242,10 @@
     <t>1301,1301,1301</t>
   </si>
   <si>
-    <t>400,580,800</t>
+    <t>13001,13001,13001</t>
+  </si>
+  <si>
+    <t>4000,580,800</t>
   </si>
   <si>
     <t>100,100,100</t>
@@ -293,7 +302,10 @@
     <t>1304,1304,1304</t>
   </si>
   <si>
-    <t>300,420,580</t>
+    <t>13004,13004,13004</t>
+  </si>
+  <si>
+    <t>3000,420,580</t>
   </si>
   <si>
     <t>1000,1000,1000</t>
@@ -344,7 +356,7 @@
     <t>2309,2309,2309</t>
   </si>
   <si>
-    <t>400,400,400</t>
+    <t>4000,400,400</t>
   </si>
   <si>
     <t>10,10,10</t>
@@ -363,6 +375,9 @@
   </si>
   <si>
     <t>1399,1399,1399</t>
+  </si>
+  <si>
+    <t>13999,13999,13999</t>
   </si>
   <si>
     <t>2000,2000,2000</t>
@@ -1363,8 +1378,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AD9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <dimension ref="A1:AE9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1375,25 +1390,25 @@
     <col min="7" max="7" width="37" customWidth="1"/>
     <col min="8" max="8" width="35" customWidth="1"/>
     <col min="9" max="9" width="44" customWidth="1"/>
-    <col min="10" max="10" width="40" customWidth="1"/>
-    <col min="11" max="13" width="24" customWidth="1"/>
-    <col min="14" max="14" width="20" customWidth="1"/>
-    <col min="15" max="16" width="22" customWidth="1"/>
-    <col min="17" max="18" width="18" customWidth="1"/>
-    <col min="19" max="19" width="11" customWidth="1"/>
-    <col min="20" max="20" width="20" customWidth="1"/>
-    <col min="21" max="21" width="26" customWidth="1"/>
-    <col min="22" max="22" width="22" customWidth="1"/>
-    <col min="23" max="23" width="8" customWidth="1"/>
-    <col min="24" max="24" width="16" customWidth="1"/>
-    <col min="25" max="26" width="36" customWidth="1"/>
-    <col min="27" max="27" width="30" customWidth="1"/>
-    <col min="28" max="28" width="28" customWidth="1"/>
-    <col min="29" max="29" width="41" customWidth="1"/>
-    <col min="30" max="30" width="42" customWidth="1"/>
+    <col min="10" max="11" width="40" customWidth="1"/>
+    <col min="12" max="14" width="24" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="16" max="17" width="22" customWidth="1"/>
+    <col min="18" max="19" width="18" customWidth="1"/>
+    <col min="20" max="20" width="11" customWidth="1"/>
+    <col min="21" max="21" width="20" customWidth="1"/>
+    <col min="22" max="22" width="26" customWidth="1"/>
+    <col min="23" max="23" width="22" customWidth="1"/>
+    <col min="24" max="24" width="8" customWidth="1"/>
+    <col min="25" max="25" width="16" customWidth="1"/>
+    <col min="26" max="27" width="36" customWidth="1"/>
+    <col min="28" max="28" width="30" customWidth="1"/>
+    <col min="29" max="29" width="28" customWidth="1"/>
+    <col min="30" max="30" width="41" customWidth="1"/>
+    <col min="31" max="31" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30">
+    <row r="1" spans="1:31">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1416,20 +1431,21 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="1"/>
       <c r="U1" s="2"/>
       <c r="V1" s="2"/>
-      <c r="W1" s="1"/>
+      <c r="W1" s="2"/>
       <c r="X1" s="1"/>
-      <c r="Y1" s="2"/>
+      <c r="Y1" s="1"/>
       <c r="Z1" s="2"/>
       <c r="AA1" s="2"/>
       <c r="AB1" s="2"/>
-      <c r="AC1" s="1"/>
-      <c r="AD1" s="2"/>
+      <c r="AC1" s="2"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="2"/>
     </row>
-    <row r="2" spans="1:30">
+    <row r="2" spans="1:31">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1482,10 +1498,10 @@
       <c r="R2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="S2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="T2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="U2" s="2" t="s">
@@ -1494,13 +1510,13 @@
       <c r="V2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="W2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="X2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y2" s="2" t="s">
+      <c r="Y2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="Z2" s="2" t="s">
@@ -1512,203 +1528,212 @@
       <c r="AB2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AC2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AD2" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="AE2" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="3" spans="1:30">
+    <row r="3" spans="1:31">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>33</v>
       </c>
       <c r="L3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="AA3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="AB3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="AC3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Z3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AA3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AC3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AD3" s="2" t="s">
-        <v>35</v>
+      <c r="AD3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:30">
+    <row r="4" ht="28.8" spans="1:31">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="S4" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>54</v>
       </c>
+      <c r="T4" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="U4" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="W4" s="1" t="s">
         <v>57</v>
       </c>
+      <c r="W4" s="2" t="s">
+        <v>58</v>
+      </c>
       <c r="X4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y4" s="2" t="s">
         <v>59</v>
       </c>
+      <c r="Y4" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="Z4" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AA4" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AB4" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AC4" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AD4" s="2" t="s">
+      <c r="AC4" s="2" t="s">
         <v>64</v>
       </c>
+      <c r="AD4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE4" s="2" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30">
+    <row r="5" ht="15" customHeight="1" spans="1:31">
       <c r="A5" s="1"/>
       <c r="B5" s="1">
         <v>1</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E5" s="1">
         <v>2</v>
@@ -1717,86 +1742,89 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="S5" s="1">
+        <v>78</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="T5" s="1">
         <v>3</v>
       </c>
-      <c r="T5" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="U5" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="W5" s="1">
-        <v>0</v>
+        <v>80</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="X5" s="1">
         <v>0</v>
       </c>
-      <c r="Y5" s="2" t="s">
-        <v>79</v>
+      <c r="Y5" s="1">
+        <v>0</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AC5" s="1">
+        <v>84</v>
+      </c>
+      <c r="AC5" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD5" s="1">
         <v>2</v>
       </c>
-      <c r="AD5" s="2" t="s">
-        <v>83</v>
+      <c r="AE5" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30">
+    <row r="6" ht="15" customHeight="1" spans="1:31">
       <c r="A6" s="1"/>
       <c r="B6" s="1">
         <v>4</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E6" s="1">
         <v>2</v>
@@ -1805,86 +1833,89 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="S6" s="1">
+        <v>98</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="T6" s="1">
         <v>3</v>
       </c>
-      <c r="T6" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="U6" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="W6" s="1">
-        <v>0</v>
+        <v>101</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>102</v>
       </c>
       <c r="X6" s="1">
         <v>0</v>
       </c>
-      <c r="Y6" s="2" t="s">
-        <v>99</v>
+      <c r="Y6" s="1">
+        <v>0</v>
       </c>
       <c r="Z6" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="AB6" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="AC6" s="1">
+        <v>105</v>
+      </c>
+      <c r="AC6" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="AD6" s="1">
         <v>2</v>
       </c>
-      <c r="AD6" s="2" t="s">
-        <v>83</v>
+      <c r="AE6" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30">
+    <row r="7" ht="15" customHeight="1" spans="1:31">
       <c r="A7" s="1"/>
       <c r="B7" s="1">
         <v>9</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E7" s="1">
         <v>2</v>
@@ -1893,86 +1924,89 @@
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>70</v>
+        <v>109</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="S7" s="1">
+        <v>112</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="T7" s="1">
         <v>3</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="U7" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="W7" s="1">
-        <v>0</v>
+        <v>101</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="X7" s="1">
         <v>0</v>
       </c>
-      <c r="Y7" s="2" t="s">
-        <v>79</v>
+      <c r="Y7" s="1">
+        <v>0</v>
       </c>
       <c r="Z7" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AA7" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AB7" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AC7" s="1">
+        <v>84</v>
+      </c>
+      <c r="AC7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD7" s="1">
         <v>2</v>
       </c>
-      <c r="AD7" s="2" t="s">
-        <v>83</v>
+      <c r="AE7" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30">
+    <row r="8" ht="15" customHeight="1" spans="1:31">
       <c r="A8" s="1"/>
       <c r="B8" s="1">
         <v>9999</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E8" s="1">
         <v>1</v>
@@ -1983,78 +2017,81 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>70</v>
+        <v>117</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="S8" s="1">
+        <v>81</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="T8" s="1">
         <v>0</v>
       </c>
-      <c r="T8" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="U8" s="2" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="W8" s="1">
-        <v>0</v>
+        <v>101</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="X8" s="1">
         <v>0</v>
       </c>
-      <c r="Y8" s="2"/>
-      <c r="Z8" s="2" t="s">
-        <v>113</v>
-      </c>
+      <c r="Y8" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="2"/>
       <c r="AA8" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB8" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="AC8" s="1">
+        <v>118</v>
+      </c>
+      <c r="AC8" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="AD8" s="1">
         <v>3</v>
       </c>
-      <c r="AD8" s="2" t="s">
-        <v>83</v>
+      <c r="AE8" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30">
+    <row r="9" ht="15" customHeight="1" spans="1:31">
       <c r="A9" s="1"/>
       <c r="B9" s="1">
         <v>1001</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E9" s="1">
         <v>3</v>
@@ -2065,67 +2102,70 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>66</v>
+        <v>121</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="O9" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="T9" s="1">
+        <v>0</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="W9" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="S9" s="1">
-        <v>0</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="U9" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="V9" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="W9" s="1">
-        <v>0</v>
       </c>
       <c r="X9" s="1">
         <v>0</v>
       </c>
-      <c r="Y9" s="2"/>
-      <c r="Z9" s="2" t="s">
-        <v>113</v>
-      </c>
+      <c r="Y9" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="2"/>
       <c r="AA9" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB9" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="AC9" s="1">
+        <v>118</v>
+      </c>
+      <c r="AC9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="AD9" s="1">
         <v>0</v>
       </c>
-      <c r="AD9" s="2"/>
+      <c r="AE9" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>